<commit_message>
added packaging options, jar candles options, added discovery set, fixed home page fragrance images
</commit_message>
<xml_diff>
--- a/data/mysaa_products.xlsx
+++ b/data/mysaa_products.xlsx
@@ -1088,9 +1088,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1112,9 +1110,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -1199,9 +1195,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
@@ -1220,7 +1214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="2"/>
@@ -1359,7 +1353,6 @@
           <t>220 ml</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -1437,7 +1430,6 @@
           <t>120 ml</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -1515,7 +1507,6 @@
           <t>60 ml</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -1593,7 +1584,6 @@
           <t>Combo</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -1671,7 +1661,6 @@
           <t>Curated set</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
@@ -1749,7 +1738,6 @@
           <t>220 ml</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -1827,7 +1815,6 @@
           <t>120 ml</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -1905,7 +1892,6 @@
           <t>60 ml</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -1983,7 +1969,6 @@
           <t>Combo</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2061,7 +2046,6 @@
           <t>Curated set</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
@@ -2139,7 +2123,6 @@
           <t>220 ml</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2217,7 +2200,6 @@
           <t>120 ml</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2295,7 +2277,6 @@
           <t>60 ml</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2373,7 +2354,6 @@
           <t>Combo</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2451,7 +2431,6 @@
           <t>Curated set</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
@@ -2529,7 +2508,6 @@
           <t>220 ml</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2607,7 +2585,6 @@
           <t>120 ml</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2685,7 +2662,6 @@
           <t>60 ml</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2763,7 +2739,6 @@
           <t>Combo</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2841,7 +2816,6 @@
           <t>Curated set</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
@@ -2919,7 +2893,6 @@
           <t>220 ml</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -2997,7 +2970,6 @@
           <t>120 ml</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -3075,7 +3047,6 @@
           <t>60 ml</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -3153,7 +3124,6 @@
           <t>Combo</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -3231,7 +3201,6 @@
           <t>Curated set</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
@@ -3309,7 +3278,6 @@
           <t>220 ml</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -3387,7 +3355,6 @@
           <t>120 ml</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -3465,7 +3432,6 @@
           <t>60 ml</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -3538,8 +3504,6 @@
       <c r="E30" t="n">
         <v>350</v>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -3612,8 +3576,6 @@
       <c r="E31" t="n">
         <v>0</v>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
@@ -3659,6 +3621,84 @@
       <c r="R31" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/gift-hampers/03-lifestyle.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>discover-set-6-shot-glass-candles</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Mysaa Rituals Discover Set</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>discovery-set</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>all-fragrances</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>6 × 60 ml</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Discover Set presentation box</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>All six Mysaa Rituals fragrances in six 60 ml shot glass jar candles.</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>A discovery set featuring all six Mysaa Rituals fragrances — six 60 ml shot glass jar candles designed to let you experience the full fragrance collection in one beautiful set.</t>
+        </is>
+      </c>
+      <c r="L32" t="b">
+        <v>0</v>
+      </c>
+      <c r="M32" t="b">
+        <v>1</v>
+      </c>
+      <c r="N32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O32" t="b">
+        <v>1</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>assets/catalogue/all-fragrances/discovery-set/01-discover-set.jpg</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>assets/catalogue/all-fragrances/discovery-set/02-gulab-ki-chitthi.jpg</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>assets/catalogue/all-fragrances/discovery-set/03-dhoop-chandan.jpg</t>
         </is>
       </c>
     </row>
@@ -3906,7 +3946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="5"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="2"/>
@@ -4033,6 +4073,26 @@
         </is>
       </c>
       <c r="D6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>discovery-set</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Discovery Set</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>6 × 60 ml shot glass candles</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
aaj ke new changes
</commit_message>
<xml_diff>
--- a/data/mysaa_products.xlsx
+++ b/data/mysaa_products.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="18600" windowHeight="6800" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,195 +14,32 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="165" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="166" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="167" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="23">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <b val="1"/>
-      <color rgb="FF7A1420"/>
+      <color rgb="007A1420"/>
       <sz val="14"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color rgb="FF800080"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color rgb="FF9C6500"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color theme="0"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -210,198 +48,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF7A1420"/>
-        <bgColor rgb="FF7A1420"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="007A1420"/>
+        <bgColor rgb="007A1420"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -409,311 +61,19 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="6"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1066,6 +426,7 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -1076,17 +437,20 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A20"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.5" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>MYSAA RITUALS — Product Data Workbook</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1109,6 +473,9 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -1140,7 +507,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   wax-melts, gift-hampers. A product's categorySlug must match one</t>
+          <t xml:space="preserve">   mold-candles, wax-melts, gift-hampers, discovery-set. A product's categorySlug must match one</t>
         </is>
       </c>
     </row>
@@ -1192,6 +559,9 @@
           <t xml:space="preserve">   will update the live site automatically within a minute or two.</t>
         </is>
       </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1211,116 +581,140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S32"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.5"/>
+  <dimension ref="A1:V39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="37" customWidth="1" min="1" max="2"/>
-    <col width="19" customWidth="1" min="3" max="4"/>
+    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="50" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="50" customWidth="1" min="16" max="18"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="50" customWidth="1" min="20" max="20"/>
+    <col width="50" customWidth="1" min="21" max="21"/>
+    <col width="50" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>categorySlug</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>fragranceSlug</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>mrp</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>discountPercent</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>moq</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>optionValues</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>volume</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>materials</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>packaging</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>shortDescription</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>about</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>bestseller</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>isNew</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>customizable</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>image1</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>image2</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>image3</t>
         </is>
@@ -1334,7 +728,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gulab Ki Chitthi Hero Jar Candle</t>
+          <t>Gulab Ki Chitthi Signature</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1348,59 +742,67 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>899</v>
+        <v>998.75</v>
       </c>
       <c r="F2" t="n">
         <v>799</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
         <is>
           <t>220 ml</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Gulab Ki Chitthi in our hero jar candle.</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals hero jar candle in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M2" t="b">
-        <v>0</v>
-      </c>
-      <c r="N2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O2" t="b">
-        <v>1</v>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Gulab Ki Chitthi in our signature.</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R2" t="b">
+        <v>1</v>
+      </c>
+      <c r="S2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -1414,7 +816,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gulab Ki Chitthi Wide Jar Candle</t>
+          <t>Gulab Ki Chitthi Everyday Ritual</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1428,59 +830,67 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>699</v>
+        <v>645.88</v>
       </c>
       <c r="F3" t="n">
         <v>549</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="n">
+        <v>15</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
         <is>
           <t>120 ml</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Gulab Ki Chitthi in our wide jar candle.</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals wide jar candle in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M3" t="b">
-        <v>0</v>
-      </c>
-      <c r="N3" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" t="b">
-        <v>1</v>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Gulab Ki Chitthi in our everyday ritual.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals everyday ritual in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q3" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" t="b">
+        <v>1</v>
+      </c>
+      <c r="S3" t="b">
+        <v>1</v>
+      </c>
+      <c r="T3" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -1494,7 +904,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Gulab Ki Chitthi Shot Glass Candle</t>
+          <t>Gulab Ki Chitthi Mini Ritual</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1508,59 +918,67 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>399</v>
+        <v>332.22</v>
       </c>
       <c r="F4" t="n">
         <v>299</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>60 ml</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Gulab Ki Chitthi in our shot glass candle.</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals shot glass candle in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M4" t="b">
-        <v>0</v>
-      </c>
-      <c r="N4" t="b">
-        <v>0</v>
-      </c>
-      <c r="O4" t="b">
-        <v>1</v>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Gulab Ki Chitthi in our mini ritual.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals mini ritual in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P4" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q4" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" t="b">
+        <v>1</v>
+      </c>
+      <c r="S4" t="b">
+        <v>1</v>
+      </c>
+      <c r="T4" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -1587,57 +1005,68 @@
           <t>gulab-ki-chitthi</t>
         </is>
       </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
       <c r="F5" t="n">
         <v>350</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Gulab Ki Chitthi in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O5" t="b">
-        <v>1</v>
-      </c>
       <c r="P5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q5" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="b">
+        <v>0</v>
+      </c>
+      <c r="R5" t="b">
+        <v>1</v>
+      </c>
+      <c r="S5" t="b">
+        <v>1</v>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -1664,57 +1093,68 @@
           <t>gulab-ki-chitthi</t>
         </is>
       </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Curated set</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Gulab Ki Chitthi in our gift hamper.</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M6" t="b">
-        <v>0</v>
-      </c>
-      <c r="N6" t="b">
-        <v>0</v>
-      </c>
-      <c r="O6" t="b">
-        <v>1</v>
-      </c>
       <c r="P6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q6" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="b">
+        <v>0</v>
+      </c>
+      <c r="R6" t="b">
+        <v>1</v>
+      </c>
+      <c r="S6" t="b">
+        <v>1</v>
+      </c>
+      <c r="T6" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -1728,7 +1168,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dhoop &amp; Chandan Hero Jar Candle</t>
+          <t>Dhoop &amp; Chandan Signature</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1742,59 +1182,67 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>899</v>
+        <v>998.75</v>
       </c>
       <c r="F7" t="n">
         <v>799</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="n">
+        <v>20</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
         <is>
           <t>220 ml</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Dhoop &amp; Chandan in our hero jar candle.</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals hero jar candle in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M7" t="b">
-        <v>0</v>
-      </c>
-      <c r="N7" t="b">
-        <v>0</v>
-      </c>
-      <c r="O7" t="b">
-        <v>1</v>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Dhoop &amp; Chandan in our signature.</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q7" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="b">
+        <v>0</v>
+      </c>
+      <c r="R7" t="b">
+        <v>1</v>
+      </c>
+      <c r="S7" t="b">
+        <v>1</v>
+      </c>
+      <c r="T7" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -1808,7 +1256,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dhoop &amp; Chandan Wide Jar Candle</t>
+          <t>Dhoop &amp; Chandan Everyday Ritual</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1822,59 +1270,67 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>699</v>
+        <v>645.88</v>
       </c>
       <c r="F8" t="n">
         <v>549</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="n">
+        <v>15</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
         <is>
           <t>120 ml</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Dhoop &amp; Chandan in our wide jar candle.</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals wide jar candle in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M8" t="b">
-        <v>0</v>
-      </c>
-      <c r="N8" t="b">
-        <v>0</v>
-      </c>
-      <c r="O8" t="b">
-        <v>1</v>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Dhoop &amp; Chandan in our everyday ritual.</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals everyday ritual in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P8" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q8" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="b">
+        <v>0</v>
+      </c>
+      <c r="R8" t="b">
+        <v>1</v>
+      </c>
+      <c r="S8" t="b">
+        <v>1</v>
+      </c>
+      <c r="T8" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -1888,7 +1344,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dhoop &amp; Chandan Shot Glass Candle</t>
+          <t>Dhoop &amp; Chandan Mini Ritual</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1902,59 +1358,67 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>399</v>
+        <v>332.22</v>
       </c>
       <c r="F9" t="n">
         <v>299</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
         <is>
           <t>60 ml</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Dhoop &amp; Chandan in our shot glass candle.</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals shot glass candle in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M9" t="b">
-        <v>0</v>
-      </c>
-      <c r="N9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O9" t="b">
-        <v>1</v>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Dhoop &amp; Chandan in our mini ritual.</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals mini ritual in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q9" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="b">
+        <v>0</v>
+      </c>
+      <c r="R9" t="b">
+        <v>1</v>
+      </c>
+      <c r="S9" t="b">
+        <v>1</v>
+      </c>
+      <c r="T9" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -1981,57 +1445,68 @@
           <t>dhoop-chandan</t>
         </is>
       </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
       <c r="F10" t="n">
         <v>350</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Dhoop &amp; Chandan in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M10" t="b">
-        <v>0</v>
-      </c>
-      <c r="N10" t="b">
-        <v>0</v>
-      </c>
-      <c r="O10" t="b">
-        <v>1</v>
-      </c>
       <c r="P10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q10" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="b">
+        <v>0</v>
+      </c>
+      <c r="R10" t="b">
+        <v>1</v>
+      </c>
+      <c r="S10" t="b">
+        <v>1</v>
+      </c>
+      <c r="T10" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -2058,57 +1533,68 @@
           <t>dhoop-chandan</t>
         </is>
       </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
         <is>
           <t>Curated set</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Dhoop &amp; Chandan in our gift hamper.</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M11" t="b">
-        <v>0</v>
-      </c>
-      <c r="N11" t="b">
-        <v>0</v>
-      </c>
-      <c r="O11" t="b">
-        <v>1</v>
-      </c>
       <c r="P11" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q11" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="b">
+        <v>0</v>
+      </c>
+      <c r="R11" t="b">
+        <v>1</v>
+      </c>
+      <c r="S11" t="b">
+        <v>1</v>
+      </c>
+      <c r="T11" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -2122,7 +1608,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Gajre Ka Shringar Hero Jar Candle</t>
+          <t>Gajre Ka Shringar Signature</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2136,59 +1622,67 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>899</v>
+        <v>998.75</v>
       </c>
       <c r="F12" t="n">
         <v>799</v>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" t="n">
+        <v>20</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
         <is>
           <t>220 ml</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Gajre Ka Shringar in our hero jar candle.</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals hero jar candle in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M12" t="b">
-        <v>0</v>
-      </c>
-      <c r="N12" t="b">
-        <v>0</v>
-      </c>
-      <c r="O12" t="b">
-        <v>1</v>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Gajre Ka Shringar in our signature.</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P12" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q12" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="b">
+        <v>0</v>
+      </c>
+      <c r="R12" t="b">
+        <v>1</v>
+      </c>
+      <c r="S12" t="b">
+        <v>1</v>
+      </c>
+      <c r="T12" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -2202,7 +1696,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Gajre Ka Shringar Wide Jar Candle</t>
+          <t>Gajre Ka Shringar Everyday Ritual</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2216,59 +1710,67 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>699</v>
+        <v>645.88</v>
       </c>
       <c r="F13" t="n">
         <v>549</v>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" t="n">
+        <v>15</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
         <is>
           <t>120 ml</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Gajre Ka Shringar in our wide jar candle.</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals wide jar candle in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M13" t="b">
-        <v>0</v>
-      </c>
-      <c r="N13" t="b">
-        <v>0</v>
-      </c>
-      <c r="O13" t="b">
-        <v>1</v>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Gajre Ka Shringar in our everyday ritual.</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals everyday ritual in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P13" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q13" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="b">
+        <v>0</v>
+      </c>
+      <c r="R13" t="b">
+        <v>1</v>
+      </c>
+      <c r="S13" t="b">
+        <v>1</v>
+      </c>
+      <c r="T13" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -2282,7 +1784,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Gajre Ka Shringar Shot Glass Candle</t>
+          <t>Gajre Ka Shringar Mini Ritual</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2296,59 +1798,67 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>399</v>
+        <v>332.22</v>
       </c>
       <c r="F14" t="n">
         <v>299</v>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" t="n">
+        <v>10</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
         <is>
           <t>60 ml</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Gajre Ka Shringar in our shot glass candle.</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals shot glass candle in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M14" t="b">
-        <v>0</v>
-      </c>
-      <c r="N14" t="b">
-        <v>0</v>
-      </c>
-      <c r="O14" t="b">
-        <v>1</v>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Gajre Ka Shringar in our mini ritual.</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals mini ritual in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P14" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q14" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="b">
+        <v>0</v>
+      </c>
+      <c r="R14" t="b">
+        <v>1</v>
+      </c>
+      <c r="S14" t="b">
+        <v>1</v>
+      </c>
+      <c r="T14" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -2375,57 +1885,68 @@
           <t>gajre-ka-shringar</t>
         </is>
       </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
       <c r="F15" t="n">
         <v>350</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Gajre Ka Shringar in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M15" t="b">
-        <v>0</v>
-      </c>
-      <c r="N15" t="b">
-        <v>0</v>
-      </c>
-      <c r="O15" t="b">
-        <v>1</v>
-      </c>
       <c r="P15" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q15" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="b">
+        <v>0</v>
+      </c>
+      <c r="R15" t="b">
+        <v>1</v>
+      </c>
+      <c r="S15" t="b">
+        <v>1</v>
+      </c>
+      <c r="T15" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -2452,57 +1973,68 @@
           <t>gajre-ka-shringar</t>
         </is>
       </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
         <is>
           <t>Curated set</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>Gajre Ka Shringar in our gift hamper.</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M16" t="b">
-        <v>0</v>
-      </c>
-      <c r="N16" t="b">
-        <v>0</v>
-      </c>
-      <c r="O16" t="b">
-        <v>1</v>
-      </c>
       <c r="P16" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q16" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="b">
+        <v>0</v>
+      </c>
+      <c r="R16" t="b">
+        <v>1</v>
+      </c>
+      <c r="S16" t="b">
+        <v>1</v>
+      </c>
+      <c r="T16" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -2516,7 +2048,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Madhuban Hero Jar Candle</t>
+          <t>Madhuban Signature</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2530,59 +2062,67 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>899</v>
+        <v>998.75</v>
       </c>
       <c r="F17" t="n">
         <v>799</v>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" t="n">
+        <v>20</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
         <is>
           <t>220 ml</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Madhuban in our hero jar candle.</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals hero jar candle in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M17" t="b">
-        <v>0</v>
-      </c>
-      <c r="N17" t="b">
-        <v>0</v>
-      </c>
-      <c r="O17" t="b">
-        <v>1</v>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Madhuban in our signature.</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P17" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q17" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="b">
+        <v>0</v>
+      </c>
+      <c r="R17" t="b">
+        <v>1</v>
+      </c>
+      <c r="S17" t="b">
+        <v>1</v>
+      </c>
+      <c r="T17" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -2596,7 +2136,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Madhuban Wide Jar Candle</t>
+          <t>Madhuban Everyday Ritual</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2610,59 +2150,67 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>699</v>
+        <v>645.88</v>
       </c>
       <c r="F18" t="n">
         <v>549</v>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" t="n">
+        <v>15</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
         <is>
           <t>120 ml</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Madhuban in our wide jar candle.</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals wide jar candle in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M18" t="b">
-        <v>0</v>
-      </c>
-      <c r="N18" t="b">
-        <v>0</v>
-      </c>
-      <c r="O18" t="b">
-        <v>1</v>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Madhuban in our everyday ritual.</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals everyday ritual in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P18" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q18" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="b">
+        <v>0</v>
+      </c>
+      <c r="R18" t="b">
+        <v>1</v>
+      </c>
+      <c r="S18" t="b">
+        <v>1</v>
+      </c>
+      <c r="T18" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="V18" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -2676,7 +2224,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Madhuban Shot Glass Candle</t>
+          <t>Madhuban Mini Ritual</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2690,59 +2238,67 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>399</v>
+        <v>332.22</v>
       </c>
       <c r="F19" t="n">
         <v>299</v>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
         <is>
           <t>60 ml</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Madhuban in our shot glass candle.</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals shot glass candle in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M19" t="b">
-        <v>0</v>
-      </c>
-      <c r="N19" t="b">
-        <v>0</v>
-      </c>
-      <c r="O19" t="b">
-        <v>1</v>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Madhuban in our mini ritual.</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals mini ritual in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P19" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q19" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="b">
+        <v>0</v>
+      </c>
+      <c r="R19" t="b">
+        <v>1</v>
+      </c>
+      <c r="S19" t="b">
+        <v>1</v>
+      </c>
+      <c r="T19" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="V19" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -2769,57 +2325,68 @@
           <t>madhuban</t>
         </is>
       </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
       <c r="F20" t="n">
         <v>350</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>Madhuban in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M20" t="b">
-        <v>0</v>
-      </c>
-      <c r="N20" t="b">
-        <v>0</v>
-      </c>
-      <c r="O20" t="b">
-        <v>1</v>
-      </c>
       <c r="P20" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q20" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="b">
+        <v>0</v>
+      </c>
+      <c r="R20" t="b">
+        <v>1</v>
+      </c>
+      <c r="S20" t="b">
+        <v>1</v>
+      </c>
+      <c r="T20" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="V20" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -2846,57 +2413,68 @@
           <t>madhuban</t>
         </is>
       </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
         <is>
           <t>Curated set</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>Madhuban in our gift hamper.</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M21" t="b">
-        <v>0</v>
-      </c>
-      <c r="N21" t="b">
-        <v>0</v>
-      </c>
-      <c r="O21" t="b">
-        <v>1</v>
-      </c>
       <c r="P21" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q21" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="b">
+        <v>0</v>
+      </c>
+      <c r="R21" t="b">
+        <v>1</v>
+      </c>
+      <c r="S21" t="b">
+        <v>1</v>
+      </c>
+      <c r="T21" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="V21" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -2910,7 +2488,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Raat Ki Rani Hero Jar Candle</t>
+          <t>Raat Ki Rani Signature</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2924,59 +2502,67 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>899</v>
+        <v>998.75</v>
       </c>
       <c r="F22" t="n">
         <v>799</v>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" t="n">
+        <v>20</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
         <is>
           <t>220 ml</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Raat Ki Rani in our hero jar candle.</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals hero jar candle in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M22" t="b">
-        <v>0</v>
-      </c>
-      <c r="N22" t="b">
-        <v>0</v>
-      </c>
-      <c r="O22" t="b">
-        <v>1</v>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Raat Ki Rani in our signature.</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P22" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q22" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="b">
+        <v>0</v>
+      </c>
+      <c r="R22" t="b">
+        <v>1</v>
+      </c>
+      <c r="S22" t="b">
+        <v>1</v>
+      </c>
+      <c r="T22" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr">
+      <c r="V22" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -2990,7 +2576,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Raat Ki Rani Wide Jar Candle</t>
+          <t>Raat Ki Rani Everyday Ritual</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3004,59 +2590,67 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>699</v>
+        <v>645.88</v>
       </c>
       <c r="F23" t="n">
         <v>549</v>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" t="n">
+        <v>15</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
         <is>
           <t>120 ml</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Raat Ki Rani in our wide jar candle.</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals wide jar candle in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M23" t="b">
-        <v>0</v>
-      </c>
-      <c r="N23" t="b">
-        <v>0</v>
-      </c>
-      <c r="O23" t="b">
-        <v>1</v>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Raat Ki Rani in our everyday ritual.</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals everyday ritual in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P23" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q23" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="b">
+        <v>0</v>
+      </c>
+      <c r="R23" t="b">
+        <v>1</v>
+      </c>
+      <c r="S23" t="b">
+        <v>1</v>
+      </c>
+      <c r="T23" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="V23" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -3070,7 +2664,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Raat Ki Rani Shot Glass Candle</t>
+          <t>Raat Ki Rani Mini Ritual</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3084,59 +2678,67 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>399</v>
+        <v>332.22</v>
       </c>
       <c r="F24" t="n">
         <v>299</v>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" t="n">
+        <v>10</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
         <is>
           <t>60 ml</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Raat Ki Rani in our shot glass candle.</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals shot glass candle in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M24" t="b">
-        <v>0</v>
-      </c>
-      <c r="N24" t="b">
-        <v>0</v>
-      </c>
-      <c r="O24" t="b">
-        <v>1</v>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Raat Ki Rani in our mini ritual.</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals mini ritual in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P24" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q24" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="b">
+        <v>0</v>
+      </c>
+      <c r="R24" t="b">
+        <v>1</v>
+      </c>
+      <c r="S24" t="b">
+        <v>1</v>
+      </c>
+      <c r="T24" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="U24" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="V24" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -3163,57 +2765,68 @@
           <t>raat-ki-rani</t>
         </is>
       </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
       <c r="F25" t="n">
         <v>350</v>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
         <is>
           <t>Combo</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>Raat Ki Rani in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M25" t="b">
-        <v>0</v>
-      </c>
-      <c r="N25" t="b">
-        <v>0</v>
-      </c>
-      <c r="O25" t="b">
-        <v>1</v>
-      </c>
       <c r="P25" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q25" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="b">
+        <v>0</v>
+      </c>
+      <c r="R25" t="b">
+        <v>1</v>
+      </c>
+      <c r="S25" t="b">
+        <v>1</v>
+      </c>
+      <c r="T25" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr">
+      <c r="V25" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -3240,57 +2853,68 @@
           <t>raat-ki-rani</t>
         </is>
       </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
       <c r="F26" t="n">
         <v>0</v>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
         <is>
           <t>Curated set</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
         <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>Raat Ki Rani in our gift hamper.</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M26" t="b">
-        <v>0</v>
-      </c>
-      <c r="N26" t="b">
-        <v>0</v>
-      </c>
-      <c r="O26" t="b">
-        <v>1</v>
-      </c>
       <c r="P26" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q26" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="b">
+        <v>0</v>
+      </c>
+      <c r="R26" t="b">
+        <v>1</v>
+      </c>
+      <c r="S26" t="b">
+        <v>1</v>
+      </c>
+      <c r="T26" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="U26" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="V26" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -3304,7 +2928,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Saanjh Hero Jar Candle</t>
+          <t>Saanjh Signature</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3318,59 +2942,67 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>899</v>
+        <v>998.75</v>
       </c>
       <c r="F27" t="n">
         <v>799</v>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" t="n">
+        <v>20</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
         <is>
           <t>220 ml</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Saanjh in our hero jar candle.</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals hero jar candle in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M27" t="b">
-        <v>0</v>
-      </c>
-      <c r="N27" t="b">
-        <v>0</v>
-      </c>
-      <c r="O27" t="b">
-        <v>1</v>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Saanjh in our signature.</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P27" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q27" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="b">
+        <v>0</v>
+      </c>
+      <c r="R27" t="b">
+        <v>1</v>
+      </c>
+      <c r="S27" t="b">
+        <v>1</v>
+      </c>
+      <c r="T27" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr">
+      <c r="V27" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -3384,7 +3016,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Saanjh Wide Jar Candle</t>
+          <t>Saanjh Everyday Ritual</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3398,59 +3030,67 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>699</v>
+        <v>645.88</v>
       </c>
       <c r="F28" t="n">
         <v>549</v>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" t="n">
+        <v>15</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
         <is>
           <t>120 ml</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Saanjh in our wide jar candle.</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals wide jar candle in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M28" t="b">
-        <v>0</v>
-      </c>
-      <c r="N28" t="b">
-        <v>1</v>
-      </c>
-      <c r="O28" t="b">
-        <v>1</v>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Saanjh in our everyday ritual.</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals everyday ritual in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P28" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q28" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="b">
+        <v>1</v>
+      </c>
+      <c r="R28" t="b">
+        <v>1</v>
+      </c>
+      <c r="S28" t="b">
+        <v>1</v>
+      </c>
+      <c r="T28" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="U28" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
+      <c r="V28" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -3464,7 +3104,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Saanjh Shot Glass Candle</t>
+          <t>Saanjh Mini Ritual</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3478,59 +3118,67 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>399</v>
+        <v>332.22</v>
       </c>
       <c r="F29" t="n">
         <v>299</v>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" t="n">
+        <v>10</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
         <is>
           <t>60 ml</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Saanjh in our shot glass candle.</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals shot glass candle in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="M29" t="b">
-        <v>0</v>
-      </c>
-      <c r="N29" t="b">
-        <v>0</v>
-      </c>
-      <c r="O29" t="b">
-        <v>1</v>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Saanjh in our mini ritual.</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals mini ritual in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="P29" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q29" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="b">
+        <v>0</v>
+      </c>
+      <c r="R29" t="b">
+        <v>1</v>
+      </c>
+      <c r="S29" t="b">
+        <v>1</v>
+      </c>
+      <c r="T29" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="V29" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -3557,52 +3205,64 @@
           <t>saanjh</t>
         </is>
       </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
       <c r="F30" t="n">
         <v>350</v>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>Saanjh in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M30" t="b">
-        <v>0</v>
-      </c>
-      <c r="N30" t="b">
-        <v>0</v>
-      </c>
-      <c r="O30" t="b">
-        <v>1</v>
-      </c>
       <c r="P30" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q30" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="b">
+        <v>0</v>
+      </c>
+      <c r="R30" t="b">
+        <v>1</v>
+      </c>
+      <c r="S30" t="b">
+        <v>1</v>
+      </c>
+      <c r="T30" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="U30" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S30" t="inlineStr">
+      <c r="V30" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -3629,52 +3289,64 @@
           <t>saanjh</t>
         </is>
       </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>Saanjh in our gift hamper.</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="M31" t="b">
-        <v>0</v>
-      </c>
-      <c r="N31" t="b">
-        <v>0</v>
-      </c>
-      <c r="O31" t="b">
-        <v>1</v>
-      </c>
       <c r="P31" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q31" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="b">
+        <v>0</v>
+      </c>
+      <c r="R31" t="b">
+        <v>1</v>
+      </c>
+      <c r="S31" t="b">
+        <v>1</v>
+      </c>
+      <c r="T31" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="U31" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr">
+      <c r="V31" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -3688,7 +3360,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Mysaa Rituals Discover Set</t>
+          <t>Mysaa Rituals Discovery Set</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3702,63 +3374,602 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1999</v>
+        <v>2123.75</v>
       </c>
       <c r="F32" t="n">
         <v>1699</v>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" t="n">
+        <v>20</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
         <is>
           <t>6 × 60 ml</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>Discover Set presentation box</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>All six Mysaa Rituals fragrances in six 60 ml shot glass jar candles.</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>A discovery set featuring all six Mysaa Rituals fragrances — six 60 ml shot glass jar candles designed to let you experience the full fragrance collection in one beautiful set.</t>
-        </is>
-      </c>
-      <c r="M32" t="b">
-        <v>0</v>
-      </c>
-      <c r="N32" t="b">
-        <v>1</v>
-      </c>
-      <c r="O32" t="b">
-        <v>0</v>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>All six Mysaa Rituals fragrances in six 60 ml Mini Ritual candles.</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>A complete discovery of all six Mysaa Rituals fragrances, presented as six 60 ml Mini Ritual candles.</t>
+        </is>
       </c>
       <c r="P32" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q32" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="b">
+        <v>1</v>
+      </c>
+      <c r="R32" t="b">
+        <v>0</v>
+      </c>
+      <c r="S32" t="b">
+        <v>1</v>
+      </c>
+      <c r="T32" t="inlineStr">
         <is>
           <t>assets/catalogue/all-fragrances/discovery-set/01-discover-set.jpg</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
+      <c r="U32" t="inlineStr">
         <is>
           <t>assets/catalogue/all-fragrances/discovery-set/02-gulab-ki-chitthi.jpg</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr">
+      <c r="V32" t="inlineStr">
         <is>
           <t>assets/catalogue/all-fragrances/discovery-set/03-dhoop-chandan.jpg</t>
         </is>
       </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>gulab-ki-chitthi-grand-ritual</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Gulab Ki Chitthi Grand Ritual</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>grand-ritual</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>gulab-ki-chitthi</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Mysaa Rituals signature packaging</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Gulab Ki Chitthi in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Gulab Ki Chitthi fragrance. Designed for statement gifting and elevated spaces.</t>
+        </is>
+      </c>
+      <c r="P33" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="b">
+        <v>1</v>
+      </c>
+      <c r="R33" t="b">
+        <v>1</v>
+      </c>
+      <c r="S33" t="b">
+        <v>1</v>
+      </c>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>dhoop-chandan-grand-ritual</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Dhoop &amp; Chandan Grand Ritual</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>grand-ritual</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>dhoop-chandan</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Mysaa Rituals signature packaging</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Dhoop &amp; Chandan in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Dhoop &amp; Chandan fragrance. Designed for statement gifting and elevated spaces.</t>
+        </is>
+      </c>
+      <c r="P34" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="b">
+        <v>1</v>
+      </c>
+      <c r="R34" t="b">
+        <v>1</v>
+      </c>
+      <c r="S34" t="b">
+        <v>1</v>
+      </c>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>gajre-ka-shringar-grand-ritual</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Gajre Ka Shringar Grand Ritual</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>grand-ritual</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>gajre-ka-shringar</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Mysaa Rituals signature packaging</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Gajre Ka Shringar in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Gajre Ka Shringar fragrance. Designed for statement gifting and elevated spaces.</t>
+        </is>
+      </c>
+      <c r="P35" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="b">
+        <v>1</v>
+      </c>
+      <c r="R35" t="b">
+        <v>1</v>
+      </c>
+      <c r="S35" t="b">
+        <v>1</v>
+      </c>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>madhuban-grand-ritual</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Madhuban Grand Ritual</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>grand-ritual</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>madhuban</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Mysaa Rituals signature packaging</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Madhuban in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Madhuban fragrance. Designed for statement gifting and elevated spaces.</t>
+        </is>
+      </c>
+      <c r="P36" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="b">
+        <v>1</v>
+      </c>
+      <c r="R36" t="b">
+        <v>1</v>
+      </c>
+      <c r="S36" t="b">
+        <v>1</v>
+      </c>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>raat-ki-rani-grand-ritual</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Raat Ki Rani Grand Ritual</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>grand-ritual</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>raat-ki-rani</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Mysaa Rituals signature packaging</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Raat Ki Rani in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Raat Ki Rani fragrance. Designed for statement gifting and elevated spaces.</t>
+        </is>
+      </c>
+      <c r="P37" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="b">
+        <v>1</v>
+      </c>
+      <c r="R37" t="b">
+        <v>1</v>
+      </c>
+      <c r="S37" t="b">
+        <v>1</v>
+      </c>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>saanjh-grand-ritual</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Saanjh Grand Ritual</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>grand-ritual</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>saanjh</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Mysaa Rituals signature packaging</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Saanjh in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Saanjh fragrance. Designed for statement gifting and elevated spaces.</t>
+        </is>
+      </c>
+      <c r="P38" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="b">
+        <v>1</v>
+      </c>
+      <c r="R38" t="b">
+        <v>1</v>
+      </c>
+      <c r="S38" t="b">
+        <v>1</v>
+      </c>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>mold-candles</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Mold Candles</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>mold-candles</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>6</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Daisy|Rose|Carnation|Cactus|Tortoise|Laddu|Chakli</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>MOQ 6 pieces</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Hand-poured wax candle</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Mysaa Rituals signature packaging</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Choose from Daisy, Rose, Carnation, Cactus, Tortoise, Laddu or Chakli moulds. Minimum order 6 pieces.</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>A playful collection of handcrafted mould candles. Select one mould style for a minimum batch of 6 pieces.</t>
+        </is>
+      </c>
+      <c r="P39" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="b">
+        <v>1</v>
+      </c>
+      <c r="R39" t="b">
+        <v>1</v>
+      </c>
+      <c r="S39" t="b">
+        <v>1</v>
+      </c>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3772,9 +3983,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="2"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
     <col width="43" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
@@ -3782,32 +3994,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>mood</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
@@ -3916,7 +4128,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Raat ki Rani, rose, deep florals</t>
+          <t>Jasmine, rose</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4004,31 +4216,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="5"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>subtitle</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
@@ -4042,7 +4255,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hero Jar Candle</t>
+          <t>Signature</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4062,7 +4275,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wide Jar Candle</t>
+          <t>Everyday Ritual</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4082,7 +4295,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Shot Glass Candle</t>
+          <t>Mini Ritual</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4147,10 +4360,50 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6 × 60 ml shot glass candles</t>
+          <t>6 × 60 ml Mini Ritual candles</t>
         </is>
       </c>
       <c r="D7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>grand-ritual</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Grand Ritual</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>450 ml · 3-wick luxury appearance</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>mold-candles</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mold Candles</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MOQ 6 pieces · choose your shape</t>
+        </is>
+      </c>
+      <c r="D9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4165,20 +4418,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.5"/>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>key</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>value</t>
         </is>
@@ -4214,7 +4467,7 @@
           <t>whatsapp</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>919919115120</t>
         </is>
@@ -4226,7 +4479,7 @@
           <t>phone</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>+91 9919115120</t>
         </is>
@@ -4238,7 +4491,7 @@
           <t>email</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>mysaarituals@gmail.com</t>
         </is>
@@ -4304,10 +4557,140 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>feedbackUrl</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://forms.cloud.microsoft/r/6S4JFC1WaX?origin=QRCode</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>feedbackQr</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>./assets/feedback-qr.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>connectQr</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>./assets/connect-qr.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>giftWrapEnabled</t>
+        </is>
+      </c>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>giftWrapCharge</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>festivalBannerEnabled</t>
+        </is>
+      </c>
+      <c r="B17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>festivalBannerEyebrow</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Upcoming · Navratri &amp; Dussehra</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>festivalBannerTitle</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Light up the season. Gift a little warmth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>festivalBannerText</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Bring home thoughtful candles and gifts for Navratri, Dussehra and the festive celebrations ahead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>festivalBannerButtonText</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Shop the Festive Collection</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>festivalBannerCategory</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>festivals-celebrations</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>festivalBannerImage</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" display="mysaarituals@gmail.com" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added details page for molds
</commit_message>
<xml_diff>
--- a/data/mysaa_products.xlsx
+++ b/data/mysaa_products.xlsx
@@ -507,7 +507,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   mold-candles, wax-melts, gift-hampers, discovery-set. A product's categorySlug must match one</t>
+          <t xml:space="preserve">   mold-candles, wax-melts, gift-hampers, discovery-set, grand-ritual. A product's categorySlug must match one</t>
         </is>
       </c>
     </row>
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:X39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -592,20 +592,22 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="50" customWidth="1" min="14" max="14"/>
-    <col width="50" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="35" customWidth="1" min="15" max="15"/>
+    <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="50" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="50" customWidth="1" min="20" max="20"/>
-    <col width="50" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
     <col width="50" customWidth="1" min="22" max="22"/>
+    <col width="50" customWidth="1" min="23" max="23"/>
+    <col width="50" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -651,70 +653,80 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
+          <t>availability</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>occasionSlugs</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
           <t>optionValues</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>volume</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>materials</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>packaging</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>shortDescription</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>about</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>bestseller</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>isNew</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>customizable</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>image1</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>image2</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>image3</t>
         </is>
@@ -728,7 +740,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Gulab Ki Chitthi Signature</t>
+          <t>Gulab Ki Chitthi Signature Ritual</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -742,7 +754,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>998.75</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="n">
         <v>799</v>
@@ -754,55 +766,57 @@
         <v>1</v>
       </c>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>220 ml</t>
-        </is>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
+          <t>220 ml</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Gulab Ki Chitthi in our signature.</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals signature in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="P2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="b">
-        <v>0</v>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Gulab Ki Chitthi in our signature ritual.</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature ritual in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="R2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T2" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U2" t="b">
+        <v>1</v>
+      </c>
+      <c r="V2" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -830,7 +844,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>645.88</v>
+        <v>650</v>
       </c>
       <c r="F3" t="n">
         <v>549</v>
@@ -842,55 +856,57 @@
         <v>1</v>
       </c>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>120 ml</t>
-        </is>
-      </c>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
+          <t>120 ml</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Gulab Ki Chitthi in our everyday ritual.</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>A Mysaa Rituals everyday ritual in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P3" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="b">
-        <v>0</v>
-      </c>
       <c r="R3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="b">
-        <v>1</v>
-      </c>
-      <c r="T3" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T3" t="b">
+        <v>1</v>
+      </c>
+      <c r="U3" t="b">
+        <v>1</v>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -918,7 +934,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>332.22</v>
+        <v>350</v>
       </c>
       <c r="F4" t="n">
         <v>299</v>
@@ -930,55 +946,57 @@
         <v>1</v>
       </c>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>60 ml</t>
-        </is>
-      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Gulab Ki Chitthi in our mini ritual.</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>A Mysaa Rituals mini ritual in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P4" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="b">
-        <v>0</v>
-      </c>
       <c r="R4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" t="b">
-        <v>1</v>
-      </c>
-      <c r="T4" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T4" t="b">
+        <v>1</v>
+      </c>
+      <c r="U4" t="b">
+        <v>1</v>
+      </c>
+      <c r="V4" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -1017,56 +1035,62 @@
       <c r="H5" t="n">
         <v>1</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Combo</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>out-of-stock</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
+          <t>Combo</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Gulab Ki Chitthi in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P5" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="b">
-        <v>0</v>
-      </c>
       <c r="R5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S5" t="b">
-        <v>1</v>
-      </c>
-      <c r="T5" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T5" t="b">
+        <v>1</v>
+      </c>
+      <c r="U5" t="b">
+        <v>1</v>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -1108,53 +1132,59 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Curated set</t>
+          <t>weddings-return-gifts</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
+          <t>Curated set</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Gulab Ki Chitthi in our gift hamper.</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Gulab Ki Chitthi fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P6" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="b">
-        <v>0</v>
-      </c>
       <c r="R6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6" t="b">
-        <v>1</v>
-      </c>
-      <c r="T6" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T6" t="b">
+        <v>1</v>
+      </c>
+      <c r="U6" t="b">
+        <v>1</v>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>assets/catalogue/gulab-ki-chitthi/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -1168,7 +1198,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dhoop &amp; Chandan Signature</t>
+          <t>Dhoop &amp; Chandan Signature Ritual</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1182,7 +1212,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>998.75</v>
+        <v>1000</v>
       </c>
       <c r="F7" t="n">
         <v>799</v>
@@ -1194,55 +1224,57 @@
         <v>1</v>
       </c>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>220 ml</t>
-        </is>
-      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
+          <t>220 ml</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Dhoop &amp; Chandan in our signature.</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals signature in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="P7" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="b">
-        <v>0</v>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Dhoop &amp; Chandan in our signature ritual.</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature ritual in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="b">
-        <v>1</v>
-      </c>
-      <c r="T7" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T7" t="b">
+        <v>1</v>
+      </c>
+      <c r="U7" t="b">
+        <v>1</v>
+      </c>
+      <c r="V7" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -1270,7 +1302,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>645.88</v>
+        <v>650</v>
       </c>
       <c r="F8" t="n">
         <v>549</v>
@@ -1282,55 +1314,57 @@
         <v>1</v>
       </c>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>120 ml</t>
-        </is>
-      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
+          <t>120 ml</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Dhoop &amp; Chandan in our everyday ritual.</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>A Mysaa Rituals everyday ritual in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P8" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="b">
-        <v>0</v>
-      </c>
       <c r="R8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" t="b">
-        <v>1</v>
-      </c>
-      <c r="T8" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T8" t="b">
+        <v>1</v>
+      </c>
+      <c r="U8" t="b">
+        <v>1</v>
+      </c>
+      <c r="V8" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -1358,7 +1392,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>332.22</v>
+        <v>350</v>
       </c>
       <c r="F9" t="n">
         <v>299</v>
@@ -1370,55 +1404,57 @@
         <v>1</v>
       </c>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>60 ml</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>Dhoop &amp; Chandan in our mini ritual.</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>A Mysaa Rituals mini ritual in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P9" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="b">
-        <v>0</v>
-      </c>
       <c r="R9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S9" t="b">
-        <v>1</v>
-      </c>
-      <c r="T9" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T9" t="b">
+        <v>1</v>
+      </c>
+      <c r="U9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V9" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -1457,56 +1493,62 @@
       <c r="H10" t="n">
         <v>1</v>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Combo</t>
-        </is>
-      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>out-of-stock</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
+          <t>Combo</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Dhoop &amp; Chandan in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P10" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="b">
-        <v>0</v>
-      </c>
       <c r="R10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" t="b">
-        <v>1</v>
-      </c>
-      <c r="T10" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T10" t="b">
+        <v>1</v>
+      </c>
+      <c r="U10" t="b">
+        <v>1</v>
+      </c>
+      <c r="V10" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="X10" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -1548,53 +1590,59 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Curated set</t>
+          <t>festivals-celebrations</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
+          <t>Curated set</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>Dhoop &amp; Chandan in our gift hamper.</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Dhoop &amp; Chandan fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P11" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="b">
-        <v>0</v>
-      </c>
       <c r="R11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="b">
-        <v>1</v>
-      </c>
-      <c r="T11" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T11" t="b">
+        <v>1</v>
+      </c>
+      <c r="U11" t="b">
+        <v>1</v>
+      </c>
+      <c r="V11" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>assets/catalogue/dhoop-chandan/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -1608,7 +1656,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Gajre Ka Shringar Signature</t>
+          <t>Gajre Ka Shringar Signature Ritual</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1622,7 +1670,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>998.75</v>
+        <v>1000</v>
       </c>
       <c r="F12" t="n">
         <v>799</v>
@@ -1634,55 +1682,57 @@
         <v>1</v>
       </c>
       <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>220 ml</t>
-        </is>
-      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
+          <t>220 ml</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Gajre Ka Shringar in our signature.</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals signature in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="P12" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="b">
-        <v>0</v>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Gajre Ka Shringar in our signature ritual.</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature ritual in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="R12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S12" t="b">
-        <v>1</v>
-      </c>
-      <c r="T12" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T12" t="b">
+        <v>1</v>
+      </c>
+      <c r="U12" t="b">
+        <v>1</v>
+      </c>
+      <c r="V12" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="X12" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -1710,7 +1760,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>645.88</v>
+        <v>650</v>
       </c>
       <c r="F13" t="n">
         <v>549</v>
@@ -1722,55 +1772,57 @@
         <v>1</v>
       </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>120 ml</t>
-        </is>
-      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
+          <t>120 ml</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Gajre Ka Shringar in our everyday ritual.</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>A Mysaa Rituals everyday ritual in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P13" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="b">
-        <v>0</v>
-      </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="b">
-        <v>1</v>
-      </c>
-      <c r="T13" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T13" t="b">
+        <v>1</v>
+      </c>
+      <c r="U13" t="b">
+        <v>1</v>
+      </c>
+      <c r="V13" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -1798,7 +1850,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>332.22</v>
+        <v>350</v>
       </c>
       <c r="F14" t="n">
         <v>299</v>
@@ -1810,55 +1862,57 @@
         <v>1</v>
       </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>60 ml</t>
-        </is>
-      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Gajre Ka Shringar in our mini ritual.</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>A Mysaa Rituals mini ritual in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P14" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="b">
-        <v>0</v>
-      </c>
       <c r="R14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" t="b">
-        <v>1</v>
-      </c>
-      <c r="T14" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T14" t="b">
+        <v>1</v>
+      </c>
+      <c r="U14" t="b">
+        <v>1</v>
+      </c>
+      <c r="V14" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -1897,56 +1951,62 @@
       <c r="H15" t="n">
         <v>1</v>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Combo</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>out-of-stock</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
+          <t>Combo</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Gajre Ka Shringar in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P15" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="b">
-        <v>0</v>
-      </c>
       <c r="R15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" t="b">
-        <v>1</v>
-      </c>
-      <c r="T15" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T15" t="b">
+        <v>1</v>
+      </c>
+      <c r="U15" t="b">
+        <v>1</v>
+      </c>
+      <c r="V15" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -1988,53 +2048,59 @@
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Curated set</t>
+          <t>weddings-return-gifts</t>
         </is>
       </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
+          <t>Curated set</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>Gajre Ka Shringar in our gift hamper.</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Gajre Ka Shringar fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P16" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="b">
-        <v>0</v>
-      </c>
       <c r="R16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="b">
-        <v>1</v>
-      </c>
-      <c r="T16" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T16" t="b">
+        <v>1</v>
+      </c>
+      <c r="U16" t="b">
+        <v>1</v>
+      </c>
+      <c r="V16" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>assets/catalogue/gajre-ka-shringar/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -2048,7 +2114,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Madhuban Signature</t>
+          <t>Madhuban Signature Ritual</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2062,7 +2128,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>998.75</v>
+        <v>1000</v>
       </c>
       <c r="F17" t="n">
         <v>799</v>
@@ -2074,55 +2140,57 @@
         <v>1</v>
       </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>220 ml</t>
-        </is>
-      </c>
+      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
+          <t>220 ml</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Madhuban in our signature.</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals signature in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="P17" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="b">
-        <v>0</v>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Madhuban in our signature ritual.</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature ritual in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="R17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S17" t="b">
-        <v>1</v>
-      </c>
-      <c r="T17" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T17" t="b">
+        <v>1</v>
+      </c>
+      <c r="U17" t="b">
+        <v>1</v>
+      </c>
+      <c r="V17" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -2150,7 +2218,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>645.88</v>
+        <v>650</v>
       </c>
       <c r="F18" t="n">
         <v>549</v>
@@ -2162,55 +2230,57 @@
         <v>1</v>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>120 ml</t>
-        </is>
-      </c>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
+          <t>120 ml</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>Madhuban in our everyday ritual.</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>A Mysaa Rituals everyday ritual in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P18" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="b">
-        <v>0</v>
-      </c>
       <c r="R18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S18" t="b">
-        <v>1</v>
-      </c>
-      <c r="T18" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T18" t="b">
+        <v>1</v>
+      </c>
+      <c r="U18" t="b">
+        <v>1</v>
+      </c>
+      <c r="V18" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="W18" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -2238,7 +2308,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>332.22</v>
+        <v>350</v>
       </c>
       <c r="F19" t="n">
         <v>299</v>
@@ -2250,55 +2320,57 @@
         <v>1</v>
       </c>
       <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>60 ml</t>
-        </is>
-      </c>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>Madhuban in our mini ritual.</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>A Mysaa Rituals mini ritual in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P19" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q19" t="b">
-        <v>0</v>
-      </c>
       <c r="R19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S19" t="b">
-        <v>1</v>
-      </c>
-      <c r="T19" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T19" t="b">
+        <v>1</v>
+      </c>
+      <c r="U19" t="b">
+        <v>1</v>
+      </c>
+      <c r="V19" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -2337,56 +2409,62 @@
       <c r="H20" t="n">
         <v>1</v>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Combo</t>
-        </is>
-      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>out-of-stock</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
+          <t>Combo</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>Madhuban in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P20" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="b">
-        <v>0</v>
-      </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="b">
-        <v>1</v>
-      </c>
-      <c r="T20" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T20" t="b">
+        <v>1</v>
+      </c>
+      <c r="U20" t="b">
+        <v>1</v>
+      </c>
+      <c r="V20" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -2428,53 +2506,59 @@
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Curated set</t>
+          <t>festivals-celebrations</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
+          <t>Curated set</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>Madhuban in our gift hamper.</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Madhuban fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P21" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q21" t="b">
-        <v>0</v>
-      </c>
       <c r="R21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S21" t="b">
-        <v>1</v>
-      </c>
-      <c r="T21" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T21" t="b">
+        <v>1</v>
+      </c>
+      <c r="U21" t="b">
+        <v>1</v>
+      </c>
+      <c r="V21" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>assets/catalogue/madhuban/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -2488,7 +2572,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Raat Ki Rani Signature</t>
+          <t>Raat Ki Rani Signature Ritual</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2502,7 +2586,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>998.75</v>
+        <v>1000</v>
       </c>
       <c r="F22" t="n">
         <v>799</v>
@@ -2514,55 +2598,57 @@
         <v>1</v>
       </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>220 ml</t>
-        </is>
-      </c>
+      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
+          <t>220 ml</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Raat Ki Rani in our signature.</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals signature in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="P22" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q22" t="b">
-        <v>0</v>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Raat Ki Rani in our signature ritual.</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature ritual in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="R22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S22" t="b">
-        <v>1</v>
-      </c>
-      <c r="T22" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T22" t="b">
+        <v>1</v>
+      </c>
+      <c r="U22" t="b">
+        <v>1</v>
+      </c>
+      <c r="V22" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="W22" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -2590,7 +2676,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>645.88</v>
+        <v>650</v>
       </c>
       <c r="F23" t="n">
         <v>549</v>
@@ -2602,55 +2688,57 @@
         <v>1</v>
       </c>
       <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>120 ml</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
+          <t>120 ml</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>Raat Ki Rani in our everyday ritual.</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>A Mysaa Rituals everyday ritual in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P23" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q23" t="b">
-        <v>0</v>
-      </c>
       <c r="R23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="b">
-        <v>1</v>
-      </c>
-      <c r="T23" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T23" t="b">
+        <v>1</v>
+      </c>
+      <c r="U23" t="b">
+        <v>1</v>
+      </c>
+      <c r="V23" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="W23" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -2678,7 +2766,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>332.22</v>
+        <v>350</v>
       </c>
       <c r="F24" t="n">
         <v>299</v>
@@ -2690,55 +2778,57 @@
         <v>1</v>
       </c>
       <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>60 ml</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="P24" t="inlineStr">
         <is>
           <t>Raat Ki Rani in our mini ritual.</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>A Mysaa Rituals mini ritual in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P24" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="b">
-        <v>0</v>
-      </c>
       <c r="R24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S24" t="b">
-        <v>1</v>
-      </c>
-      <c r="T24" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T24" t="b">
+        <v>1</v>
+      </c>
+      <c r="U24" t="b">
+        <v>1</v>
+      </c>
+      <c r="V24" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="W24" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -2777,56 +2867,62 @@
       <c r="H25" t="n">
         <v>1</v>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Combo</t>
-        </is>
-      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>out-of-stock</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
+          <t>Combo</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="P25" t="inlineStr">
         <is>
           <t>Raat Ki Rani in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P25" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q25" t="b">
-        <v>0</v>
-      </c>
       <c r="R25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S25" t="b">
-        <v>1</v>
-      </c>
-      <c r="T25" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T25" t="b">
+        <v>1</v>
+      </c>
+      <c r="U25" t="b">
+        <v>1</v>
+      </c>
+      <c r="V25" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="W25" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -2868,53 +2964,59 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Curated set</t>
+          <t>birthdays-just-because</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
+          <t>Curated set</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
           <t>Curated Mysaa Rituals gifting selection</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>Raat Ki Rani in our gift hamper.</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Raat Ki Rani fragrance. Made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P26" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q26" t="b">
-        <v>0</v>
-      </c>
       <c r="R26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S26" t="b">
-        <v>1</v>
-      </c>
-      <c r="T26" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T26" t="b">
+        <v>1</v>
+      </c>
+      <c r="U26" t="b">
+        <v>1</v>
+      </c>
+      <c r="V26" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="W26" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>assets/catalogue/raat-ki-rani/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -2928,7 +3030,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Saanjh Signature</t>
+          <t>Saanjh Signature Ritual</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2942,7 +3044,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>998.75</v>
+        <v>1000</v>
       </c>
       <c r="F27" t="n">
         <v>799</v>
@@ -2954,55 +3056,57 @@
         <v>1</v>
       </c>
       <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>220 ml</t>
-        </is>
-      </c>
+      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
+          <t>220 ml</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Saanjh in our signature.</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>A Mysaa Rituals signature in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
-        </is>
-      </c>
-      <c r="P27" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q27" t="b">
-        <v>0</v>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Saanjh in our signature ritual.</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>A Mysaa Rituals signature ritual in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
+        </is>
       </c>
       <c r="R27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S27" t="b">
-        <v>1</v>
-      </c>
-      <c r="T27" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T27" t="b">
+        <v>1</v>
+      </c>
+      <c r="U27" t="b">
+        <v>1</v>
+      </c>
+      <c r="V27" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/hero-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="W27" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/hero-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/hero-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -3030,7 +3134,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>645.88</v>
+        <v>650</v>
       </c>
       <c r="F28" t="n">
         <v>549</v>
@@ -3042,55 +3146,57 @@
         <v>1</v>
       </c>
       <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>120 ml</t>
-        </is>
-      </c>
+      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
+          <t>120 ml</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="P28" t="inlineStr">
         <is>
           <t>Saanjh in our everyday ritual.</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t>A Mysaa Rituals everyday ritual in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P28" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q28" t="b">
-        <v>1</v>
-      </c>
       <c r="R28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S28" t="b">
         <v>1</v>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="T28" t="b">
+        <v>1</v>
+      </c>
+      <c r="U28" t="b">
+        <v>1</v>
+      </c>
+      <c r="V28" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wide-jar-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="W28" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wide-jar-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wide-jar-candle/03-lifestyle.jpg</t>
         </is>
@@ -3118,7 +3224,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>332.22</v>
+        <v>350</v>
       </c>
       <c r="F29" t="n">
         <v>299</v>
@@ -3130,55 +3236,57 @@
         <v>1</v>
       </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>60 ml</t>
-        </is>
-      </c>
+      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
+          <t>60 ml</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="P29" t="inlineStr">
         <is>
           <t>Saanjh in our mini ritual.</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>A Mysaa Rituals mini ritual in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P29" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q29" t="b">
-        <v>0</v>
-      </c>
       <c r="R29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S29" t="b">
-        <v>1</v>
-      </c>
-      <c r="T29" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T29" t="b">
+        <v>1</v>
+      </c>
+      <c r="U29" t="b">
+        <v>1</v>
+      </c>
+      <c r="V29" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/shot-glass-candle/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="W29" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/shot-glass-candle/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/shot-glass-candle/03-lifestyle.jpg</t>
         </is>
@@ -3217,52 +3325,58 @@
       <c r="H30" t="n">
         <v>1</v>
       </c>
-      <c r="I30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>out-of-stock</t>
+        </is>
+      </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr">
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="P30" t="inlineStr">
         <is>
           <t>Saanjh in our wax sachet combo.</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>A Mysaa Rituals wax sachet combo in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P30" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="b">
-        <v>0</v>
-      </c>
       <c r="R30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S30" t="b">
-        <v>1</v>
-      </c>
-      <c r="T30" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T30" t="b">
+        <v>1</v>
+      </c>
+      <c r="U30" t="b">
+        <v>1</v>
+      </c>
+      <c r="V30" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wax-melts/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="W30" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wax-melts/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/wax-melts/03-lifestyle.jpg</t>
         </is>
@@ -3302,51 +3416,57 @@
         <v>1</v>
       </c>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>birthdays-just-because</t>
+        </is>
+      </c>
       <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
         <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>Saanjh in our gift hamper.</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>A Mysaa Rituals gift hamper in the Saanjh fragrance — creamy vanilla softened by deep sandalwood, made for gifting, rituals and everyday moments.</t>
         </is>
       </c>
-      <c r="P31" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q31" t="b">
-        <v>0</v>
-      </c>
       <c r="R31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31" t="b">
-        <v>1</v>
-      </c>
-      <c r="T31" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="T31" t="b">
+        <v>1</v>
+      </c>
+      <c r="U31" t="b">
+        <v>1</v>
+      </c>
+      <c r="V31" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/gift-hampers/01-cover.jpg</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="W31" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/gift-hampers/02-detail.jpg</t>
         </is>
       </c>
-      <c r="V31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>assets/catalogue/saanjh/gift-hampers/03-lifestyle.jpg</t>
         </is>
@@ -3374,7 +3494,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>2123.75</v>
+        <v>2100</v>
       </c>
       <c r="F32" t="n">
         <v>1699</v>
@@ -3386,55 +3506,57 @@
         <v>1</v>
       </c>
       <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>6 × 60 ml</t>
-        </is>
-      </c>
+      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
+          <t>6 × 60 ml</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wick, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>Discover Set presentation box</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="P32" t="inlineStr">
         <is>
           <t>All six Mysaa Rituals fragrances in six 60 ml Mini Ritual candles.</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="Q32" t="inlineStr">
         <is>
           <t>A complete discovery of all six Mysaa Rituals fragrances, presented as six 60 ml Mini Ritual candles.</t>
         </is>
       </c>
-      <c r="P32" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q32" t="b">
-        <v>1</v>
-      </c>
       <c r="R32" t="b">
         <v>0</v>
       </c>
       <c r="S32" t="b">
         <v>1</v>
       </c>
-      <c r="T32" t="inlineStr">
+      <c r="T32" t="b">
+        <v>0</v>
+      </c>
+      <c r="U32" t="b">
+        <v>1</v>
+      </c>
+      <c r="V32" t="inlineStr">
         <is>
           <t>assets/catalogue/all-fragrances/discovery-set/01-discover-set.jpg</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="W32" t="inlineStr">
         <is>
           <t>assets/catalogue/all-fragrances/discovery-set/02-gulab-ki-chitthi.jpg</t>
         </is>
       </c>
-      <c r="V32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>assets/catalogue/all-fragrances/discovery-set/03-dhoop-chandan.jpg</t>
         </is>
@@ -3474,47 +3596,49 @@
         <v>1</v>
       </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>450 ml · 3 wick</t>
-        </is>
-      </c>
+      <c r="J33" t="inlineStr"/>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="P33" t="inlineStr">
         <is>
           <t>Gulab Ki Chitthi in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="Q33" t="inlineStr">
         <is>
           <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Gulab Ki Chitthi fragrance. Designed for statement gifting and elevated spaces.</t>
         </is>
       </c>
-      <c r="P33" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q33" t="b">
-        <v>1</v>
-      </c>
       <c r="R33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S33" t="b">
         <v>1</v>
       </c>
-      <c r="T33" t="inlineStr"/>
-      <c r="U33" t="inlineStr"/>
+      <c r="T33" t="b">
+        <v>1</v>
+      </c>
+      <c r="U33" t="b">
+        <v>1</v>
+      </c>
       <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3550,47 +3674,49 @@
         <v>1</v>
       </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>450 ml · 3 wick</t>
-        </is>
-      </c>
+      <c r="J34" t="inlineStr"/>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="P34" t="inlineStr">
         <is>
           <t>Dhoop &amp; Chandan in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="Q34" t="inlineStr">
         <is>
           <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Dhoop &amp; Chandan fragrance. Designed for statement gifting and elevated spaces.</t>
         </is>
       </c>
-      <c r="P34" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q34" t="b">
-        <v>1</v>
-      </c>
       <c r="R34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S34" t="b">
         <v>1</v>
       </c>
-      <c r="T34" t="inlineStr"/>
-      <c r="U34" t="inlineStr"/>
+      <c r="T34" t="b">
+        <v>1</v>
+      </c>
+      <c r="U34" t="b">
+        <v>1</v>
+      </c>
       <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3626,47 +3752,49 @@
         <v>1</v>
       </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>450 ml · 3 wick</t>
-        </is>
-      </c>
+      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="P35" t="inlineStr">
         <is>
           <t>Gajre Ka Shringar in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="Q35" t="inlineStr">
         <is>
           <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Gajre Ka Shringar fragrance. Designed for statement gifting and elevated spaces.</t>
         </is>
       </c>
-      <c r="P35" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q35" t="b">
-        <v>1</v>
-      </c>
       <c r="R35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S35" t="b">
         <v>1</v>
       </c>
-      <c r="T35" t="inlineStr"/>
-      <c r="U35" t="inlineStr"/>
+      <c r="T35" t="b">
+        <v>1</v>
+      </c>
+      <c r="U35" t="b">
+        <v>1</v>
+      </c>
       <c r="V35" t="inlineStr"/>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3702,47 +3830,49 @@
         <v>1</v>
       </c>
       <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>450 ml · 3 wick</t>
-        </is>
-      </c>
+      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="O36" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="P36" t="inlineStr">
         <is>
           <t>Madhuban in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="Q36" t="inlineStr">
         <is>
           <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Madhuban fragrance. Designed for statement gifting and elevated spaces.</t>
         </is>
       </c>
-      <c r="P36" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q36" t="b">
-        <v>1</v>
-      </c>
       <c r="R36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S36" t="b">
         <v>1</v>
       </c>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
+      <c r="T36" t="b">
+        <v>1</v>
+      </c>
+      <c r="U36" t="b">
+        <v>1</v>
+      </c>
       <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3778,47 +3908,49 @@
         <v>1</v>
       </c>
       <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>450 ml · 3 wick</t>
-        </is>
-      </c>
+      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="P37" t="inlineStr">
         <is>
           <t>Raat Ki Rani in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="Q37" t="inlineStr">
         <is>
           <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Raat Ki Rani fragrance. Designed for statement gifting and elevated spaces.</t>
         </is>
       </c>
-      <c r="P37" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q37" t="b">
-        <v>1</v>
-      </c>
       <c r="R37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S37" t="b">
         <v>1</v>
       </c>
-      <c r="T37" t="inlineStr"/>
-      <c r="U37" t="inlineStr"/>
+      <c r="T37" t="b">
+        <v>1</v>
+      </c>
+      <c r="U37" t="b">
+        <v>1</v>
+      </c>
       <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3854,47 +3986,49 @@
         <v>1</v>
       </c>
       <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>450 ml · 3 wick</t>
-        </is>
-      </c>
+      <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
+          <t>450 ml · 3 wick</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
           <t>Natural soy wax, cotton wicks, phthalate-free fragrance oils</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="P38" t="inlineStr">
         <is>
           <t>Saanjh in our Grand Ritual — a 450 ml, 3-wick luxury candle.</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="Q38" t="inlineStr">
         <is>
           <t>A luxurious 450 ml, 3-wick Mysaa Rituals Grand Ritual in the Saanjh fragrance. Designed for statement gifting and elevated spaces.</t>
         </is>
       </c>
-      <c r="P38" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q38" t="b">
-        <v>1</v>
-      </c>
       <c r="R38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S38" t="b">
         <v>1</v>
       </c>
-      <c r="T38" t="inlineStr"/>
-      <c r="U38" t="inlineStr"/>
+      <c r="T38" t="b">
+        <v>1</v>
+      </c>
+      <c r="U38" t="b">
+        <v>1</v>
+      </c>
       <c r="V38" t="inlineStr"/>
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3913,10 +4047,10 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>399</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -3926,50 +4060,56 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
+          <t>in-stock</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
           <t>Daisy|Rose|Carnation|Cactus|Tortoise|Laddu|Chakli</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>MOQ 6 pieces</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
+          <t>6 pieces minimum</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
           <t>Hand-poured wax candle</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>Mysaa Rituals signature packaging</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>Choose from Daisy, Rose, Carnation, Cactus, Tortoise, Laddu or Chakli moulds. Minimum order 6 pieces.</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>A playful collection of handcrafted mould candles. Select one mould style for a minimum batch of 6 pieces.</t>
-        </is>
-      </c>
-      <c r="P39" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q39" t="b">
-        <v>1</v>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Create a custom batch of mould candles with your choice of shape, fragrance and primary colour.</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Choose one mould shape, one Mysaa Rituals fragrance and one primary colour for your batch. Minimum order is 6 pieces. The current batch price is ₹399 for 6 pieces.</t>
+        </is>
       </c>
       <c r="R39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S39" t="b">
         <v>1</v>
       </c>
-      <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
+      <c r="T39" t="b">
+        <v>1</v>
+      </c>
+      <c r="U39" t="b">
+        <v>1</v>
+      </c>
       <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4255,7 +4395,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Signature</t>
+          <t>Signature Ritual</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4400,7 +4540,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MOQ 6 pieces · choose your shape</t>
+          <t>MOQ 6 pieces · ₹399 for 6 pieces</t>
         </is>
       </c>
       <c r="D9" t="b">

</xml_diff>